<commit_message>
Sincronizar repositório: atualizar todos os arquivos da aplicação local
- Atualizar modelos de dados
- Atualizar rotas (auth, main, cotacao, pesquisa)
- Atualizar serviços (email, utils)
- Atualizar templates HTML
- Atualizar estilos CSS e scripts JavaScript
- Atualizar dados (contas, filiais, produtos, mesorregião)
- Atualizar bancos de dados (cotacoes, users)
- Adicionar documentação de validação e históricos
- Adicionar migrações de banco de dados
- Adicionar arquivo de debug
</commit_message>
<xml_diff>
--- a/data/FILIAL - MESOREGIAO v1.xlsx
+++ b/data/FILIAL - MESOREGIAO v1.xlsx
@@ -1,20 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joseduque\Documents\Documentos\Python\Aplicacao-Cotacao-Pesquisa\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D3AACC-B54F-487E-9549-B7F051FA2EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="20370" yWindow="-3045" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$38</definedName>
+  </definedNames>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="48">
   <si>
     <t>FILIAL</t>
   </si>
@@ -28,18 +37,12 @@
     <t>300:Unidade Avançada Muzambinho</t>
   </si>
   <si>
-    <t>301:Unidade Avançada Conceição Aparecida</t>
-  </si>
-  <si>
     <t>302:Unidade Avançada Botelhos</t>
   </si>
   <si>
     <t>303:Unidade Avançada Monte Belo</t>
   </si>
   <si>
-    <t>L01:Loja Matriz</t>
-  </si>
-  <si>
     <t>L04:Loja Cabo Verde</t>
   </si>
   <si>
@@ -155,13 +158,22 @@
   </si>
   <si>
     <t>Rafael</t>
+  </si>
+  <si>
+    <t>L27:Loja Conceição Aparecida</t>
+  </si>
+  <si>
+    <t>L01:Loja Matriz Guaxupé</t>
+  </si>
+  <si>
+    <t>L25:Loja Espirito Santo do Pinhal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -224,13 +236,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -268,7 +288,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -302,6 +322,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -336,9 +357,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -511,11 +533,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="45.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -526,403 +553,415 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
         <v>39</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C20" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
         <v>39</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C21" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
         <v>39</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C22" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
         <v>39</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C23" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
         <v>39</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C24" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C25" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
         <v>39</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C26" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
         <v>39</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C27" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
         <v>39</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C28" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
         <v>40</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C30" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
         <v>40</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C31" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
         <v>40</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C32" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
         <v>40</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C33" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" t="s">
         <v>40</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C34" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
         <v>40</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C35" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
         <v>40</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C36" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
         <v>40</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C37" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" t="s">
         <v>40</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C38" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" t="s">
-        <v>41</v>
-      </c>
-      <c r="C26" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" t="s">
-        <v>41</v>
-      </c>
-      <c r="C27" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" t="s">
-        <v>42</v>
-      </c>
-      <c r="C30" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" t="s">
-        <v>42</v>
-      </c>
-      <c r="C31" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>36</v>
-      </c>
-      <c r="B35" t="s">
-        <v>42</v>
-      </c>
-      <c r="C35" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" t="s">
-        <v>42</v>
-      </c>
-      <c r="C36" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>38</v>
-      </c>
-      <c r="B37" t="s">
-        <v>42</v>
-      </c>
-      <c r="C37" t="s">
-        <v>46</v>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:C38" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: preenchimento automatico do comprador e analise dinamica de regional/analistas
Melhorias implementadas:
1. Preenchimento automático do campo comprador se o editor for de Suprimentos
2. Script de migração migrar_comprador.py para preenchimento retroativo do comprador
3. Mapeamento dinâmico de Analistas a partir da Mesorregião (sem switch/case)
4. Mudança de REGIONAL 7 para REGIONAL nas regras de Soja e Milho
5. Inclusão dos serviços de PDF pendentes e atualização do .gitignore
</commit_message>
<xml_diff>
--- a/data/FILIAL - MESOREGIAO v1.xlsx
+++ b/data/FILIAL - MESOREGIAO v1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joseduque\Documents\Documentos\Python\Aplicacao-Cotacao-Pesquisa\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D3AACC-B54F-487E-9549-B7F051FA2EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA7EA30-D84F-4A92-BCF2-EC265AD58F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-3045" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,23 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$38</definedName>
   </definedNames>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="44">
   <si>
     <t>FILIAL</t>
   </si>
@@ -136,30 +147,6 @@
     <t>L23:Loja Manhuaçu</t>
   </si>
   <si>
-    <t>REGIONAL - Ana Cássia</t>
-  </si>
-  <si>
-    <t>REGIONAL - Leiliele</t>
-  </si>
-  <si>
-    <t>REGIONAL - Thalles</t>
-  </si>
-  <si>
-    <t>REGIONAL - Rafael</t>
-  </si>
-  <si>
-    <t>Ana Cássia</t>
-  </si>
-  <si>
-    <t>Leiliele</t>
-  </si>
-  <si>
-    <t>Thalles</t>
-  </si>
-  <si>
-    <t>Rafael</t>
-  </si>
-  <si>
     <t>L27:Loja Conceição Aparecida</t>
   </si>
   <si>
@@ -167,6 +154,18 @@
   </si>
   <si>
     <t>L25:Loja Espirito Santo do Pinhal</t>
+  </si>
+  <si>
+    <t>Thalles da Silva Rodrigues</t>
+  </si>
+  <si>
+    <t>Rafael Lasaro Moreira da Silva</t>
+  </si>
+  <si>
+    <t>Leiliele Cristina Terra Santos</t>
+  </si>
+  <si>
+    <t>Ana Cassia Moreira Reis</t>
   </si>
 </sst>
 </file>
@@ -538,8 +537,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -557,107 +556,117 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>37</v>
+      <c r="B2" t="str">
+        <f>"REGIONAL"&amp;" "&amp;"-"&amp;" "&amp;C2</f>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" t="s">
         <v>37</v>
       </c>
+      <c r="B3" t="str">
+        <f t="shared" ref="B3:B38" si="0">"REGIONAL"&amp;" "&amp;"-"&amp;" "&amp;C3</f>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
+      </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
-        <v>37</v>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
-        <v>37</v>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>37</v>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>37</v>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>37</v>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>37</v>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Ana Cassia Moreira Reis</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>38</v>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
@@ -667,8 +676,9 @@
       <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>38</v>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C12" t="s">
         <v>42</v>
@@ -678,8 +688,9 @@
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
-        <v>38</v>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C13" t="s">
         <v>42</v>
@@ -689,8 +700,9 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
-        <v>38</v>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C14" t="s">
         <v>42</v>
@@ -700,8 +712,9 @@
       <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
-        <v>38</v>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C15" t="s">
         <v>42</v>
@@ -711,8 +724,9 @@
       <c r="A16" t="s">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
-        <v>38</v>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C16" t="s">
         <v>42</v>
@@ -722,8 +736,9 @@
       <c r="A17" t="s">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
-        <v>38</v>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C17" t="s">
         <v>42</v>
@@ -733,8 +748,9 @@
       <c r="A18" t="s">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
-        <v>38</v>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C18" t="s">
         <v>42</v>
@@ -744,8 +760,9 @@
       <c r="A19" t="s">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
-        <v>38</v>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Leiliele Cristina Terra Santos</v>
       </c>
       <c r="C19" t="s">
         <v>42</v>
@@ -755,209 +772,228 @@
       <c r="A20" t="s">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
-        <v>39</v>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
-        <v>39</v>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
-        <v>39</v>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
-        <v>39</v>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>47</v>
-      </c>
-      <c r="B24" t="s">
         <v>39</v>
       </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
+      </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
-      <c r="B25" t="s">
-        <v>39</v>
+      <c r="B25" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C25" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>24</v>
       </c>
-      <c r="B26" t="s">
-        <v>39</v>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C26" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
-      <c r="B27" t="s">
-        <v>39</v>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C27" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
-      <c r="B28" t="s">
-        <v>39</v>
+      <c r="B28" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C28" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
-      <c r="B29" t="s">
-        <v>39</v>
+      <c r="B29" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Thalles da Silva Rodrigues</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
-      <c r="B30" t="s">
-        <v>40</v>
+      <c r="B30" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C30" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>29</v>
       </c>
-      <c r="B31" t="s">
-        <v>40</v>
+      <c r="B31" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C31" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
-      <c r="B32" t="s">
-        <v>40</v>
+      <c r="B32" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C32" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
-      <c r="B33" t="s">
-        <v>40</v>
+      <c r="B33" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C33" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>32</v>
       </c>
-      <c r="B34" t="s">
-        <v>40</v>
+      <c r="B34" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C34" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>33</v>
       </c>
-      <c r="B35" t="s">
-        <v>40</v>
+      <c r="B35" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C35" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
-      <c r="B36" t="s">
-        <v>40</v>
+      <c r="B36" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C36" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>35</v>
       </c>
-      <c r="B37" t="s">
-        <v>40</v>
+      <c r="B37" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C37" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>36</v>
       </c>
-      <c r="B38" t="s">
-        <v>40</v>
+      <c r="B38" t="str">
+        <f t="shared" si="0"/>
+        <v>REGIONAL - Rafael Lasaro Moreira da Silva</v>
       </c>
       <c r="C38" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>